<commit_message>
Regenerate the sample runs with the reviewed build (same plans; report wording updates)
</commit_message>
<xml_diff>
--- a/2-unreachable-window/output/routeplan.xlsx
+++ b/2-unreachable-window/output/routeplan.xlsx
@@ -5908,7 +5908,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">placed 1415 km away (Post Office Drive Up Box, Sherwood Forest, Maryvil)</t>
+          <t xml:space="preserve">placed 1415 km away ()</t>
         </is>
       </c>
     </row>
@@ -6040,7 +6040,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">placed 1415 km away (Post Office Drive Up Box, Sherwood Forest, Maryvil)</t>
+          <t xml:space="preserve">placed 1415 km away ()</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sample runs: tidy the location-uncertain wording
</commit_message>
<xml_diff>
--- a/2-unreachable-window/output/routeplan.xlsx
+++ b/2-unreachable-window/output/routeplan.xlsx
@@ -5908,7 +5908,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">placed 1415 km away ()</t>
+          <t xml:space="preserve">placed 1415 km away (Sherwood Forest, Maryville 37802)</t>
         </is>
       </c>
     </row>
@@ -6040,7 +6040,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">placed 1415 km away ()</t>
+          <t xml:space="preserve">placed 1415 km away (Sherwood Forest, Maryville 37802)</t>
         </is>
       </c>
     </row>

</xml_diff>